<commit_message>
Rename validation columns and remove unused variable in validation process
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -475,31 +475,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.5946946216248197</v>
+        <v>-0.5717750079835704</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.6516284688864773</v>
+        <v>-0.1795421045863512</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.6230053216297051</v>
+        <v>0.5962750169702573</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1800911464940715</v>
+        <v>0.3419944247400561</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.914694621624822</v>
+        <v>-2.911775007983572</v>
       </c>
       <c r="G2" t="n">
-        <v>1.403309531113528</v>
+        <v>1.428189895413653</v>
       </c>
       <c r="H2" t="n">
-        <v>2.399616678370293</v>
+        <v>2.390301016970249</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.6971128535059242</v>
+        <v>-0.6781775752599388</v>
       </c>
       <c r="J2" t="n">
-        <v>337</v>
+        <v>327</v>
       </c>
     </row>
     <row r="3">
@@ -509,31 +509,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.2204676869716593</v>
+        <v>0.4315806297584672</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6316116277130515</v>
+        <v>0.05991888284460045</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.6300925038828984</v>
+        <v>0.1239565742687041</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4717567263645661</v>
+        <v>-0.7158433612059607</v>
       </c>
       <c r="F3" t="n">
-        <v>-3.100467686971661</v>
+        <v>-2.908419370241535</v>
       </c>
       <c r="G3" t="n">
-        <v>1.579907627713057</v>
+        <v>1.397574882844608</v>
       </c>
       <c r="H3" t="n">
-        <v>2.489307496117087</v>
+        <v>2.400672574268699</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.7390472736354289</v>
+        <v>-0.6956853612059563</v>
       </c>
       <c r="J3" t="n">
-        <v>400</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4">
@@ -543,31 +543,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.9148601668296361</v>
+        <v>-0.5001467928011645</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.7893494142866844</v>
+        <v>0.5640725824767856</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1912349171371976</v>
+        <v>0.6835266960389552</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7979684883482097</v>
+        <v>0.5684518235707359</v>
       </c>
       <c r="F4" t="n">
-        <v>-3.134860166829638</v>
+        <v>-2.940146792801166</v>
       </c>
       <c r="G4" t="n">
-        <v>1.566840585713321</v>
+        <v>1.410540582476791</v>
       </c>
       <c r="H4" t="n">
-        <v>2.523239082862791</v>
+        <v>2.437570696038943</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.7441775116517847</v>
+        <v>-0.7034841764292594</v>
       </c>
       <c r="J4" t="n">
-        <v>420</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5">
@@ -577,31 +577,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5396010834921765</v>
+        <v>0.6978715958929751</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.8616595759492278</v>
+        <v>-0.05156472196459316</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9771515115275444</v>
+        <v>0.3025463890732971</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.2072422341841613</v>
+        <v>0.2646102591326018</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.920398916507826</v>
+        <v>-3.042128404107027</v>
       </c>
       <c r="G5" t="n">
-        <v>1.431324424050781</v>
+        <v>1.545461278035416</v>
       </c>
       <c r="H5" t="n">
-        <v>2.40668951152752</v>
+        <v>2.470834389073273</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.6805342341841591</v>
+        <v>-0.7281037408673957</v>
       </c>
       <c r="J5" t="n">
-        <v>366</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6">
@@ -611,31 +611,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.2171776201063156</v>
+        <v>-0.001947876721746677</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5003050925934351</v>
+        <v>0.9197921662271851</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9470112887393436</v>
+        <v>0.1960075677785513</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7885841240651541</v>
+        <v>-0.637555760961412</v>
       </c>
       <c r="F6" t="n">
-        <v>-2.897177620106318</v>
+        <v>-3.081947876721749</v>
       </c>
       <c r="G6" t="n">
-        <v>1.424801092593442</v>
+        <v>1.561458166227191</v>
       </c>
       <c r="H6" t="n">
-        <v>2.388283288739337</v>
+        <v>2.470197567778536</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.6755898759348407</v>
+        <v>-0.7346337609614059</v>
       </c>
       <c r="J6" t="n">
-        <v>325</v>
+        <v>378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README with additional library and installation instructions; modify learning rate in perceptron.py
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -475,31 +475,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.5717750079835704</v>
+        <v>-0.1724306685857611</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.1795421045863512</v>
+        <v>-0.7557090261971233</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5962750169702573</v>
+        <v>0.6529074748976202</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3419944247400561</v>
+        <v>-0.6307767042333119</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.911775007983572</v>
+        <v>-76.67243066858576</v>
       </c>
       <c r="G2" t="n">
-        <v>1.428189895413653</v>
+        <v>38.37094097380271</v>
       </c>
       <c r="H2" t="n">
-        <v>2.390301016970249</v>
+        <v>61.77160747489508</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.6781775752599388</v>
+        <v>-18.27187670423339</v>
       </c>
       <c r="J2" t="n">
-        <v>327</v>
+        <v>407</v>
       </c>
     </row>
     <row r="3">
@@ -509,31 +509,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4315806297584672</v>
+        <v>0.1955905609051134</v>
       </c>
       <c r="C3" t="n">
-        <v>0.05991888284460045</v>
+        <v>-0.2086962331095705</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1239565742687041</v>
+        <v>0.4924343061295244</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.7158433612059607</v>
+        <v>0.2150355856462434</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.908419370241535</v>
+        <v>-77.80440943909488</v>
       </c>
       <c r="G3" t="n">
-        <v>1.397574882844608</v>
+        <v>39.05230376689018</v>
       </c>
       <c r="H3" t="n">
-        <v>2.400672574268699</v>
+        <v>62.32073430612692</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.6956853612059563</v>
+        <v>-18.51846441435386</v>
       </c>
       <c r="J3" t="n">
-        <v>344</v>
+        <v>413</v>
       </c>
     </row>
     <row r="4">
@@ -543,31 +543,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.5001467928011645</v>
+        <v>0.6597297680736613</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5640725824767856</v>
+        <v>-0.6520145357565079</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6835266960389552</v>
+        <v>0.9968318785342456</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5684518235707359</v>
+        <v>0.001349962438056407</v>
       </c>
       <c r="F4" t="n">
-        <v>-2.940146792801166</v>
+        <v>-74.84027023192634</v>
       </c>
       <c r="G4" t="n">
-        <v>1.410540582476791</v>
+        <v>36.57383546424339</v>
       </c>
       <c r="H4" t="n">
-        <v>2.437570696038943</v>
+        <v>60.85418187853192</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.7034841764292594</v>
+        <v>-17.90920003756192</v>
       </c>
       <c r="J4" t="n">
-        <v>335</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5">
@@ -577,31 +577,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6978715958929751</v>
+        <v>-0.3992941881366643</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.05156472196459316</v>
+        <v>0.7200786977576501</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3025463890732971</v>
+        <v>-0.7490750266458053</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2646102591326018</v>
+        <v>-0.524003816669623</v>
       </c>
       <c r="F5" t="n">
-        <v>-3.042128404107027</v>
+        <v>-77.89929418813666</v>
       </c>
       <c r="G5" t="n">
-        <v>1.545461278035416</v>
+        <v>39.45802869775741</v>
       </c>
       <c r="H5" t="n">
-        <v>2.470834389073273</v>
+        <v>62.86767497335158</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.7281037408673957</v>
+        <v>-18.53935381666976</v>
       </c>
       <c r="J5" t="n">
-        <v>414</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6">
@@ -611,31 +611,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.001947876721746677</v>
+        <v>-0.1939165203288522</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9197921662271851</v>
+        <v>0.3319794052917484</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1960075677785513</v>
+        <v>0.8155739255630641</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.637555760961412</v>
+        <v>0.1603498216708694</v>
       </c>
       <c r="F6" t="n">
-        <v>-3.081947876721749</v>
+        <v>-77.69391652032886</v>
       </c>
       <c r="G6" t="n">
-        <v>1.561458166227191</v>
+        <v>39.29157940529151</v>
       </c>
       <c r="H6" t="n">
-        <v>2.470197567778536</v>
+        <v>62.35652392556037</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.7346337609614059</v>
+        <v>-18.51880017832926</v>
       </c>
       <c r="J6" t="n">
-        <v>378</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update datasets and graphics with new binary files
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -475,31 +475,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.1724306685857611</v>
+        <v>-0.6087784053576126</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.7557090261971233</v>
+        <v>-0.5487445920561751</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6529074748976202</v>
+        <v>-0.4509702971087202</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.6307767042333119</v>
+        <v>-0.6868191477275809</v>
       </c>
       <c r="F2" t="n">
-        <v>-76.67243066858576</v>
+        <v>-77.60877840535761</v>
       </c>
       <c r="G2" t="n">
-        <v>38.37094097380271</v>
+        <v>39.59795540794357</v>
       </c>
       <c r="H2" t="n">
-        <v>61.77160747489508</v>
+        <v>62.51792970288872</v>
       </c>
       <c r="I2" t="n">
-        <v>-18.27187670423339</v>
+        <v>-18.55411914772773</v>
       </c>
       <c r="J2" t="n">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3">
@@ -509,31 +509,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1955905609051134</v>
+        <v>-0.3180126712154099</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.2086962331095705</v>
+        <v>-0.9733872379070954</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4924343061295244</v>
+        <v>0.4276559225054144</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2150355856462434</v>
+        <v>-0.6857942490951443</v>
       </c>
       <c r="F3" t="n">
-        <v>-77.80440943909488</v>
+        <v>-76.81801267121541</v>
       </c>
       <c r="G3" t="n">
-        <v>39.05230376689018</v>
+        <v>38.89096276209271</v>
       </c>
       <c r="H3" t="n">
-        <v>62.32073430612692</v>
+        <v>61.90860592250293</v>
       </c>
       <c r="I3" t="n">
-        <v>-18.51846441435386</v>
+        <v>-18.35049424909521</v>
       </c>
       <c r="J3" t="n">
-        <v>413</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4">
@@ -543,31 +543,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6597297680736613</v>
+        <v>0.3145186956406516</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.6520145357565079</v>
+        <v>-0.478290160122504</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9968318785342456</v>
+        <v>0.09912296400867593</v>
       </c>
       <c r="E4" t="n">
-        <v>0.001349962438056407</v>
+        <v>-0.5082964533907328</v>
       </c>
       <c r="F4" t="n">
-        <v>-74.84027023192634</v>
+        <v>-76.18548130435934</v>
       </c>
       <c r="G4" t="n">
-        <v>36.57383546424339</v>
+        <v>37.93955983987728</v>
       </c>
       <c r="H4" t="n">
-        <v>60.85418187853192</v>
+        <v>61.7157229640061</v>
       </c>
       <c r="I4" t="n">
-        <v>-17.90920003756192</v>
+        <v>-18.22004645339077</v>
       </c>
       <c r="J4" t="n">
-        <v>367</v>
+        <v>387</v>
       </c>
     </row>
     <row r="5">
@@ -577,31 +577,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.3992941881366643</v>
+        <v>0.3713214874167781</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7200786977576501</v>
+        <v>0.8901166882881113</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.7490750266458053</v>
+        <v>-0.494097025871852</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.524003816669623</v>
+        <v>0.01610989679384955</v>
       </c>
       <c r="F5" t="n">
-        <v>-77.89929418813666</v>
+        <v>-76.62867851258322</v>
       </c>
       <c r="G5" t="n">
-        <v>39.45802869775741</v>
+        <v>38.77956668828798</v>
       </c>
       <c r="H5" t="n">
-        <v>62.86767497335158</v>
+        <v>61.7482029741257</v>
       </c>
       <c r="I5" t="n">
-        <v>-18.53935381666976</v>
+        <v>-18.28854010320625</v>
       </c>
       <c r="J5" t="n">
-        <v>421</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6">
@@ -611,31 +611,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.1939165203288522</v>
+        <v>0.2049896310384283</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3319794052917484</v>
+        <v>-0.1894481802764263</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8155739255630641</v>
+        <v>0.1019709430352747</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1603498216708694</v>
+        <v>-0.8243641596641831</v>
       </c>
       <c r="F6" t="n">
-        <v>-77.69391652032886</v>
+        <v>-72.29501036896157</v>
       </c>
       <c r="G6" t="n">
-        <v>39.29157940529151</v>
+        <v>34.82670181972347</v>
       </c>
       <c r="H6" t="n">
-        <v>62.35652392556037</v>
+        <v>59.88002094303312</v>
       </c>
       <c r="I6" t="n">
-        <v>-18.51880017832926</v>
+        <v>-17.2946641596641</v>
       </c>
       <c r="J6" t="n">
-        <v>419</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add metrics calculation and confusion matrix visualization
- Implemented a new script `metricas.py` to calculate performance metrics (accuracy, sensitivity, specificity, precision) for multiple models based on validation data.
- Integrated confusion matrix generation and visualization using Matplotlib, saving the output as PNG files in the specified directory.
- Added functionality to read validation data from an Excel file and save calculated metrics back to another Excel file.
- Created confusion matrix plots for each model (Y_T1 to Y_T5) with appropriate titles and labels.
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -475,31 +475,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.6087784053576126</v>
+        <v>-0.1837631299587661</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.5487445920561751</v>
+        <v>0.9739721266802996</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.4509702971087202</v>
+        <v>0.6035382309619974</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.6868191477275809</v>
+        <v>-0.5337039703251472</v>
       </c>
       <c r="F2" t="n">
-        <v>-77.60877840535761</v>
+        <v>-71.68376312995876</v>
       </c>
       <c r="G2" t="n">
-        <v>39.59795540794357</v>
+        <v>35.31517212668024</v>
       </c>
       <c r="H2" t="n">
-        <v>62.51792970288872</v>
+        <v>59.57258823095996</v>
       </c>
       <c r="I2" t="n">
-        <v>-18.55411914772773</v>
+        <v>-16.74485397032507</v>
       </c>
       <c r="J2" t="n">
-        <v>404</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3">
@@ -509,31 +509,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.3180126712154099</v>
+        <v>0.1697095415038299</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.9733872379070954</v>
+        <v>0.5709052579259848</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4276559225054144</v>
+        <v>-0.280539538111892</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.6857942490951443</v>
+        <v>-0.5602346402173033</v>
       </c>
       <c r="F3" t="n">
-        <v>-76.81801267121541</v>
+        <v>-78.33029045849617</v>
       </c>
       <c r="G3" t="n">
-        <v>38.89096276209271</v>
+        <v>40.15410525792573</v>
       </c>
       <c r="H3" t="n">
-        <v>61.90860592250293</v>
+        <v>62.87461046188537</v>
       </c>
       <c r="I3" t="n">
-        <v>-18.35049424909521</v>
+        <v>-18.71133464021748</v>
       </c>
       <c r="J3" t="n">
-        <v>386</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4">
@@ -543,31 +543,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3145186956406516</v>
+        <v>0.7987495672431788</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.478290160122504</v>
+        <v>-0.6115962491944797</v>
       </c>
       <c r="D4" t="n">
-        <v>0.09912296400867593</v>
+        <v>-0.6530763106397008</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.5082964533907328</v>
+        <v>-0.180942356277233</v>
       </c>
       <c r="F4" t="n">
-        <v>-76.18548130435934</v>
+        <v>-79.20125043275682</v>
       </c>
       <c r="G4" t="n">
-        <v>37.93955983987728</v>
+        <v>39.93275375080523</v>
       </c>
       <c r="H4" t="n">
-        <v>61.7157229640061</v>
+        <v>63.50052368935746</v>
       </c>
       <c r="I4" t="n">
-        <v>-18.22004645339077</v>
+        <v>-18.82229235627745</v>
       </c>
       <c r="J4" t="n">
-        <v>387</v>
+        <v>456</v>
       </c>
     </row>
     <row r="5">
@@ -577,31 +577,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3713214874167781</v>
+        <v>0.4188280468880923</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8901166882881113</v>
+        <v>-0.03381883881795034</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.494097025871852</v>
+        <v>0.2959224607807047</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01610989679384955</v>
+        <v>-0.5573949544614565</v>
       </c>
       <c r="F5" t="n">
-        <v>-76.62867851258322</v>
+        <v>-76.08117195311191</v>
       </c>
       <c r="G5" t="n">
-        <v>38.77956668828798</v>
+        <v>38.76218116118189</v>
       </c>
       <c r="H5" t="n">
-        <v>61.7482029741257</v>
+        <v>61.25792246077819</v>
       </c>
       <c r="I5" t="n">
-        <v>-18.28854010320625</v>
+        <v>-18.15734495446151</v>
       </c>
       <c r="J5" t="n">
-        <v>392</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6">
@@ -611,31 +611,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.2049896310384283</v>
+        <v>0.5155928571661104</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.1894481802764263</v>
+        <v>0.6450761102754865</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1019709430352747</v>
+        <v>-0.5274020967476343</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.8243641596641831</v>
+        <v>-0.8979251239570252</v>
       </c>
       <c r="F6" t="n">
-        <v>-72.29501036896157</v>
+        <v>-72.48440714283389</v>
       </c>
       <c r="G6" t="n">
-        <v>34.82670181972347</v>
+        <v>34.96502611027542</v>
       </c>
       <c r="H6" t="n">
-        <v>59.88002094303312</v>
+        <v>60.32659790325026</v>
       </c>
       <c r="I6" t="n">
-        <v>-17.2946641596641</v>
+        <v>-17.35582512395696</v>
       </c>
       <c r="J6" t="n">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adicionando rmse mas o correto e (epocas/rmse)
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -475,31 +475,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.8993940018776851</v>
+        <v>-0.3121064540045466</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.5671174368611018</v>
+        <v>-0.3937321323789618</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6025794640985909</v>
+        <v>-0.2240696893291465</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5341975656898772</v>
+        <v>0.3779318206013891</v>
       </c>
       <c r="F2" t="n">
-        <v>-77.39939400187768</v>
+        <v>-74.81210645400455</v>
       </c>
       <c r="G2" t="n">
-        <v>38.5312325631387</v>
+        <v>37.82626786762115</v>
       </c>
       <c r="H2" t="n">
-        <v>63.02142946409599</v>
+        <v>61.13593031067143</v>
       </c>
       <c r="I2" t="n">
-        <v>-17.78070243431021</v>
+        <v>-17.93206817939811</v>
       </c>
       <c r="J2" t="n">
-        <v>411</v>
+        <v>373</v>
       </c>
     </row>
     <row r="3">
@@ -509,31 +509,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.8558668526774418</v>
+        <v>0.4030576625903037</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.7312948732123297</v>
+        <v>0.0159088579052411</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0170570877973677</v>
+        <v>-0.29905671264542</v>
       </c>
       <c r="E3" t="n">
-        <v>0.005824509799784661</v>
+        <v>0.3331008435196072</v>
       </c>
       <c r="F3" t="n">
-        <v>-71.35586685267745</v>
+        <v>-77.5969423374097</v>
       </c>
       <c r="G3" t="n">
-        <v>35.14040512678766</v>
+        <v>38.83090885790523</v>
       </c>
       <c r="H3" t="n">
-        <v>59.53924291220041</v>
+        <v>62.87594328735521</v>
       </c>
       <c r="I3" t="n">
-        <v>-16.68167549020012</v>
+        <v>-18.13689915647986</v>
       </c>
       <c r="J3" t="n">
-        <v>338</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4">
@@ -543,31 +543,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.7692650250725328</v>
+        <v>-0.9764232651296036</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0227466001338601</v>
+        <v>-0.6573537634181439</v>
       </c>
       <c r="D4" t="n">
-        <v>0.307551543087131</v>
+        <v>0.3327566628705421</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.3331931209207892</v>
+        <v>0.2575580467964433</v>
       </c>
       <c r="F4" t="n">
-        <v>-76.26926502507254</v>
+        <v>-70.4764232651296</v>
       </c>
       <c r="G4" t="n">
-        <v>38.8475466001337</v>
+        <v>34.98764623658239</v>
       </c>
       <c r="H4" t="n">
-        <v>61.54030154308462</v>
+        <v>58.88775666287081</v>
       </c>
       <c r="I4" t="n">
-        <v>-18.20899312092086</v>
+        <v>-16.52744195320317</v>
       </c>
       <c r="J4" t="n">
-        <v>383</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5">
@@ -577,31 +577,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6745369434994457</v>
+        <v>-0.9307719720252072</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5752795460876179</v>
+        <v>0.3138230740749912</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.9659638756752822</v>
+        <v>-0.5520736013563112</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.08157703560078189</v>
+        <v>0.6765634678908206</v>
       </c>
       <c r="F5" t="n">
-        <v>-77.32546305650055</v>
+        <v>-78.43077197202521</v>
       </c>
       <c r="G5" t="n">
-        <v>39.18777954608741</v>
+        <v>39.93382307407477</v>
       </c>
       <c r="H5" t="n">
-        <v>62.3459361243222</v>
+        <v>63.71292639864438</v>
       </c>
       <c r="I5" t="n">
-        <v>-18.45962703560088</v>
+        <v>-18.7534365321086</v>
       </c>
       <c r="J5" t="n">
-        <v>413</v>
+        <v>436</v>
       </c>
     </row>
     <row r="6">
@@ -611,31 +611,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06189566534786528</v>
+        <v>0.8437371874847548</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.5615239285906839</v>
+        <v>-0.2694424885627456</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.7128865945917011</v>
+        <v>-0.6688111139649371</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.9699392438197671</v>
+        <v>0.496864561622645</v>
       </c>
       <c r="F6" t="n">
-        <v>-78.43810433465214</v>
+        <v>-76.15626281251525</v>
       </c>
       <c r="G6" t="n">
-        <v>40.13317607140906</v>
+        <v>38.58055751143723</v>
       </c>
       <c r="H6" t="n">
-        <v>62.99906340540554</v>
+        <v>62.38118888603574</v>
       </c>
       <c r="I6" t="n">
-        <v>-18.66638924381997</v>
+        <v>-17.84313543837684</v>
       </c>
       <c r="J6" t="n">
-        <v>444</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizar arquivos de métricas e gráficos com novos dados e visualizações
</commit_message>
<xml_diff>
--- a/datasets/resultados.xlsx
+++ b/datasets/resultados.xlsx
@@ -475,31 +475,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.3121064540045466</v>
+        <v>0.01819747329443944</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.3937321323789618</v>
+        <v>0.9938917587359959</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.2240696893291465</v>
+        <v>-0.7364840041770273</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3779318206013891</v>
+        <v>0.5004306826689027</v>
       </c>
       <c r="F2" t="n">
-        <v>-74.81210645400455</v>
+        <v>-74.98180252670556</v>
       </c>
       <c r="G2" t="n">
-        <v>37.82626786762115</v>
+        <v>37.75889175873618</v>
       </c>
       <c r="H2" t="n">
-        <v>61.13593031067143</v>
+        <v>61.27351599582359</v>
       </c>
       <c r="I2" t="n">
-        <v>-17.93206817939811</v>
+        <v>-17.50456931733061</v>
       </c>
       <c r="J2" t="n">
-        <v>373</v>
+        <v>393</v>
       </c>
     </row>
     <row r="3">
@@ -509,31 +509,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4030576625903037</v>
+        <v>0.5144866306995655</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0159088579052411</v>
+        <v>0.783787011893027</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.29905671264542</v>
+        <v>-0.5199412232207361</v>
       </c>
       <c r="E3" t="n">
-        <v>0.3331008435196072</v>
+        <v>-0.6162432620843425</v>
       </c>
       <c r="F3" t="n">
-        <v>-77.5969423374097</v>
+        <v>-75.48551336930043</v>
       </c>
       <c r="G3" t="n">
-        <v>38.83090885790523</v>
+        <v>38.20378701189311</v>
       </c>
       <c r="H3" t="n">
-        <v>62.87594328735521</v>
+        <v>61.81505877677981</v>
       </c>
       <c r="I3" t="n">
-        <v>-18.13689915647986</v>
+        <v>-17.68624326208381</v>
       </c>
       <c r="J3" t="n">
-        <v>437</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4">
@@ -543,31 +543,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.9764232651296036</v>
+        <v>-0.3576505883523542</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.6573537634181439</v>
+        <v>-0.5138509235547604</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3327566628705421</v>
+        <v>0.01663845137182829</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2575580467964433</v>
+        <v>0.6733234112700044</v>
       </c>
       <c r="F4" t="n">
-        <v>-70.4764232651296</v>
+        <v>-77.35765058835236</v>
       </c>
       <c r="G4" t="n">
-        <v>34.98764623658239</v>
+        <v>40.17114907644518</v>
       </c>
       <c r="H4" t="n">
-        <v>58.88775666287081</v>
+        <v>63.20663845137251</v>
       </c>
       <c r="I4" t="n">
-        <v>-16.52744195320317</v>
+        <v>-18.53667658872946</v>
       </c>
       <c r="J4" t="n">
-        <v>317</v>
+        <v>422</v>
       </c>
     </row>
     <row r="5">
@@ -577,31 +577,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.9307719720252072</v>
+        <v>-0.3435242104660508</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3138230740749912</v>
+        <v>0.8123864103304723</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.5520736013563112</v>
+        <v>0.92076693396693</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6765634678908206</v>
+        <v>-0.2393854235791155</v>
       </c>
       <c r="F5" t="n">
-        <v>-78.43077197202521</v>
+        <v>-73.34352421046606</v>
       </c>
       <c r="G5" t="n">
-        <v>39.93382307407477</v>
+        <v>37.89238641033069</v>
       </c>
       <c r="H5" t="n">
-        <v>63.71292639864438</v>
+        <v>60.4707669339674</v>
       </c>
       <c r="I5" t="n">
-        <v>-18.7534365321086</v>
+        <v>-17.16938542357864</v>
       </c>
       <c r="J5" t="n">
-        <v>436</v>
+        <v>370</v>
       </c>
     </row>
     <row r="6">
@@ -611,31 +611,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8437371874847548</v>
+        <v>-0.9121749429994175</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.2694424885627456</v>
+        <v>0.8705069684634661</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.6688111139649371</v>
+        <v>-0.5673830433735316</v>
       </c>
       <c r="E6" t="n">
-        <v>0.496864561622645</v>
+        <v>0.1773759191431434</v>
       </c>
       <c r="F6" t="n">
-        <v>-76.15626281251525</v>
+        <v>-76.41217494299941</v>
       </c>
       <c r="G6" t="n">
-        <v>38.58055751143723</v>
+        <v>38.51550696846362</v>
       </c>
       <c r="H6" t="n">
-        <v>62.38118888603574</v>
+        <v>62.07761695662703</v>
       </c>
       <c r="I6" t="n">
-        <v>-17.84313543837684</v>
+        <v>-18.26262408085635</v>
       </c>
       <c r="J6" t="n">
-        <v>418</v>
+        <v>409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>